<commit_message>
Tiempos con set de 500 y 3000 registros
He medido los tiempos de ejecución con el dataset LUAD_500 y LUAD original.
El dataset de 500 que he utilizado lo he dejado en el repositorio Evamtools -> examples_for_upload
He utilizado la web de Ramón para el de 500 pero tras mas de media hora lo he dejado
</commit_message>
<xml_diff>
--- a/Claudia/tiempos_MHN.xlsx
+++ b/Claudia/tiempos_MHN.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\claud_rjfw4ak\Documents\GitHub\EvAM-Tools\Claudia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1171C508-868E-43BA-AC76-9D5F65A399A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{326BF528-8C2A-491C-A211-BC8FCCD3D056}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{FDD89A57-F735-49B2-B076-DD48DEACFA57}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="31">
   <si>
     <t>Claudia</t>
   </si>
@@ -120,6 +120,15 @@
   </si>
   <si>
     <t>LUAD_500.csv</t>
+  </si>
+  <si>
+    <t>LUAD_n12.csv</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>mas 30 min</t>
   </si>
 </sst>
 </file>
@@ -536,16 +545,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BEEB152-16CF-4E65-B7F1-9FCE82C9BF13}">
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:V25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="38.1328125" customWidth="1"/>
     <col min="2" max="5" width="10.6640625" style="1"/>
     <col min="6" max="6" width="12.53125" customWidth="1"/>
     <col min="9" max="9" width="39.265625" customWidth="1"/>
+    <col min="13" max="13" width="9.59765625" customWidth="1"/>
+    <col min="14" max="14" width="12.3984375" customWidth="1"/>
+    <col min="17" max="17" width="39.46484375" customWidth="1"/>
+    <col min="22" max="22" width="25.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:22" ht="18" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="6" t="s">
         <v>21</v>
       </c>
@@ -562,8 +575,16 @@
       <c r="L1" s="6"/>
       <c r="M1" s="6"/>
       <c r="N1" s="6"/>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="Q1" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="R1" s="6"/>
+      <c r="S1" s="6"/>
+      <c r="T1" s="6"/>
+      <c r="U1" s="6"/>
+      <c r="V1" s="6"/>
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A2" s="1"/>
       <c r="B2" s="1" t="s">
         <v>0</v>
@@ -596,8 +617,24 @@
       <c r="N2" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="Q2" s="1"/>
+      <c r="R2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -611,16 +648,31 @@
       <c r="I3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="J3" s="4"/>
+      <c r="J3" s="5">
+        <v>52.161999999999999</v>
+      </c>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
       <c r="N3" s="5">
         <f>SUM(J3:M3)/4</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.45">
+        <v>13.0405</v>
+      </c>
+      <c r="Q3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="R3" s="5">
+        <v>69.486000000000004</v>
+      </c>
+      <c r="S3" s="1"/>
+      <c r="T3" s="1"/>
+      <c r="U3" s="1"/>
+      <c r="V3" s="5">
+        <f>SUM(R3:U3)/4</f>
+        <v>17.371500000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -634,16 +686,31 @@
       <c r="I4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="J4" s="1"/>
+      <c r="J4" s="5">
+        <v>25.722000000000001</v>
+      </c>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
       <c r="N4" s="5">
-        <f t="shared" ref="N4:N25" si="1">SUM(J4:M4)/4</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.45">
+        <f t="shared" ref="N4:N18" si="1">SUM(J4:M4)/4</f>
+        <v>6.4305000000000003</v>
+      </c>
+      <c r="Q4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="R4" s="5">
+        <v>27.157</v>
+      </c>
+      <c r="S4" s="1"/>
+      <c r="T4" s="1"/>
+      <c r="U4" s="1"/>
+      <c r="V4" s="5">
+        <f t="shared" ref="V4:V18" si="2">SUM(R4:U4)/4</f>
+        <v>6.78925</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
         <v>7</v>
       </c>
@@ -657,16 +724,31 @@
       <c r="I5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="1"/>
+      <c r="J5" s="5">
+        <v>24.885999999999999</v>
+      </c>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
       <c r="N5" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.45">
+        <v>6.2214999999999998</v>
+      </c>
+      <c r="Q5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="R5" s="5">
+        <v>25.812000000000001</v>
+      </c>
+      <c r="S5" s="1"/>
+      <c r="T5" s="1"/>
+      <c r="U5" s="1"/>
+      <c r="V5" s="5">
+        <f t="shared" si="2"/>
+        <v>6.4530000000000003</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
         <v>8</v>
       </c>
@@ -680,16 +762,31 @@
       <c r="I6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J6" s="1"/>
+      <c r="J6" s="5">
+        <v>21.838999999999999</v>
+      </c>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
       <c r="N6" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.45">
+        <v>5.4597499999999997</v>
+      </c>
+      <c r="Q6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="R6" s="5">
+        <v>24.166</v>
+      </c>
+      <c r="S6" s="1"/>
+      <c r="T6" s="1"/>
+      <c r="U6" s="1"/>
+      <c r="V6" s="5">
+        <f t="shared" si="2"/>
+        <v>6.0415000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
         <v>9</v>
       </c>
@@ -703,16 +800,31 @@
       <c r="I7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="J7" s="1"/>
+      <c r="J7" s="5">
+        <v>23.576000000000001</v>
+      </c>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
       <c r="N7" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.45">
+        <v>5.8940000000000001</v>
+      </c>
+      <c r="Q7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="R7" s="5">
+        <v>26.861000000000001</v>
+      </c>
+      <c r="S7" s="1"/>
+      <c r="T7" s="1"/>
+      <c r="U7" s="1"/>
+      <c r="V7" s="5">
+        <f t="shared" si="2"/>
+        <v>6.7152500000000002</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
         <v>10</v>
       </c>
@@ -726,16 +838,31 @@
       <c r="I8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="J8" s="1"/>
+      <c r="J8" s="5">
+        <v>20.138999999999999</v>
+      </c>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
       <c r="N8" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.45">
+        <v>5.0347499999999998</v>
+      </c>
+      <c r="Q8" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="R8" s="5">
+        <v>26.922999999999998</v>
+      </c>
+      <c r="S8" s="1"/>
+      <c r="T8" s="1"/>
+      <c r="U8" s="1"/>
+      <c r="V8" s="5">
+        <f t="shared" si="2"/>
+        <v>6.7307499999999996</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
@@ -749,16 +876,31 @@
       <c r="I9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="J9" s="1"/>
+      <c r="J9" s="5">
+        <v>25.446000000000002</v>
+      </c>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
       <c r="N9" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.45">
+        <v>6.3615000000000004</v>
+      </c>
+      <c r="Q9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="R9" s="5">
+        <v>27.869</v>
+      </c>
+      <c r="S9" s="1"/>
+      <c r="T9" s="1"/>
+      <c r="U9" s="1"/>
+      <c r="V9" s="5">
+        <f t="shared" si="2"/>
+        <v>6.9672499999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
         <v>12</v>
       </c>
@@ -772,16 +914,31 @@
       <c r="I10" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="J10" s="1"/>
+      <c r="J10" s="5">
+        <v>24.556999999999999</v>
+      </c>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
       <c r="N10" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.45">
+        <v>6.1392499999999997</v>
+      </c>
+      <c r="Q10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="R10" s="5">
+        <v>27.632000000000001</v>
+      </c>
+      <c r="S10" s="1"/>
+      <c r="T10" s="1"/>
+      <c r="U10" s="1"/>
+      <c r="V10" s="5">
+        <f t="shared" si="2"/>
+        <v>6.9080000000000004</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
         <v>13</v>
       </c>
@@ -795,16 +952,31 @@
       <c r="I11" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="J11" s="1"/>
+      <c r="J11" s="5">
+        <v>24.481000000000002</v>
+      </c>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
       <c r="N11" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.45">
+        <v>6.1202500000000004</v>
+      </c>
+      <c r="Q11" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="R11" s="5">
+        <v>28.274000000000001</v>
+      </c>
+      <c r="S11" s="1"/>
+      <c r="T11" s="1"/>
+      <c r="U11" s="1"/>
+      <c r="V11" s="5">
+        <f t="shared" si="2"/>
+        <v>7.0685000000000002</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A12" s="3" t="s">
         <v>14</v>
       </c>
@@ -818,16 +990,31 @@
       <c r="I12" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="J12" s="1"/>
+      <c r="J12" s="5">
+        <v>25.128</v>
+      </c>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
       <c r="N12" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.45">
+        <v>6.282</v>
+      </c>
+      <c r="Q12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="R12" s="5">
+        <v>25.454000000000001</v>
+      </c>
+      <c r="S12" s="1"/>
+      <c r="T12" s="1"/>
+      <c r="U12" s="1"/>
+      <c r="V12" s="5">
+        <f t="shared" si="2"/>
+        <v>6.3635000000000002</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A13" s="3" t="s">
         <v>15</v>
       </c>
@@ -841,16 +1028,31 @@
       <c r="I13" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="J13" s="1"/>
+      <c r="J13" s="5">
+        <v>23.295000000000002</v>
+      </c>
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
       <c r="N13" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.45">
+        <v>5.8237500000000004</v>
+      </c>
+      <c r="Q13" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R13" s="5">
+        <v>28.919</v>
+      </c>
+      <c r="S13" s="1"/>
+      <c r="T13" s="1"/>
+      <c r="U13" s="1"/>
+      <c r="V13" s="5">
+        <f t="shared" si="2"/>
+        <v>7.2297500000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A14" s="3" t="s">
         <v>16</v>
       </c>
@@ -864,16 +1066,31 @@
       <c r="I14" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J14" s="1"/>
+      <c r="J14" s="5">
+        <v>24.623999999999999</v>
+      </c>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
       <c r="N14" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.45">
+        <v>6.1559999999999997</v>
+      </c>
+      <c r="Q14" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="R14" s="5">
+        <v>28.507000000000001</v>
+      </c>
+      <c r="S14" s="1"/>
+      <c r="T14" s="1"/>
+      <c r="U14" s="1"/>
+      <c r="V14" s="5">
+        <f t="shared" si="2"/>
+        <v>7.1267500000000004</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A15" s="3" t="s">
         <v>17</v>
       </c>
@@ -887,16 +1104,31 @@
       <c r="I15" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="J15" s="1"/>
+      <c r="J15" s="5">
+        <v>25.433</v>
+      </c>
       <c r="K15" s="1"/>
       <c r="L15" s="1"/>
       <c r="M15" s="1"/>
       <c r="N15" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.45">
+        <v>6.35825</v>
+      </c>
+      <c r="Q15" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="R15" s="5">
+        <v>26.302</v>
+      </c>
+      <c r="S15" s="1"/>
+      <c r="T15" s="1"/>
+      <c r="U15" s="1"/>
+      <c r="V15" s="5">
+        <f t="shared" si="2"/>
+        <v>6.5754999999999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A16" s="3" t="s">
         <v>18</v>
       </c>
@@ -910,16 +1142,31 @@
       <c r="I16" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J16" s="1"/>
+      <c r="J16" s="5">
+        <v>21.591999999999999</v>
+      </c>
       <c r="K16" s="1"/>
       <c r="L16" s="1"/>
       <c r="M16" s="1"/>
       <c r="N16" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.45">
+        <v>5.3979999999999997</v>
+      </c>
+      <c r="Q16" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="R16" s="5">
+        <v>28977</v>
+      </c>
+      <c r="S16" s="1"/>
+      <c r="T16" s="1"/>
+      <c r="U16" s="1"/>
+      <c r="V16" s="5">
+        <f t="shared" si="2"/>
+        <v>7244.25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A17" s="3" t="s">
         <v>19</v>
       </c>
@@ -933,16 +1180,31 @@
       <c r="I17" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J17" s="1"/>
+      <c r="J17" s="5">
+        <v>21.614999999999998</v>
+      </c>
       <c r="K17" s="1"/>
       <c r="L17" s="1"/>
       <c r="M17" s="1"/>
       <c r="N17" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.45">
+        <v>5.4037499999999996</v>
+      </c>
+      <c r="Q17" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="R17" s="5">
+        <v>27.704000000000001</v>
+      </c>
+      <c r="S17" s="1"/>
+      <c r="T17" s="1"/>
+      <c r="U17" s="1"/>
+      <c r="V17" s="5">
+        <f t="shared" si="2"/>
+        <v>6.9260000000000002</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A18" s="3" t="s">
         <v>20</v>
       </c>
@@ -956,26 +1218,47 @@
       <c r="I18" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="J18" s="1"/>
+      <c r="J18" s="5">
+        <v>23.99</v>
+      </c>
       <c r="K18" s="1"/>
       <c r="L18" s="1"/>
       <c r="M18" s="1"/>
       <c r="N18" s="5">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.45">
+        <v>5.9974999999999996</v>
+      </c>
+      <c r="Q18" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="R18" s="5">
+        <v>28.715</v>
+      </c>
+      <c r="S18" s="1"/>
+      <c r="T18" s="1"/>
+      <c r="U18" s="1"/>
+      <c r="V18" s="5">
+        <f t="shared" si="2"/>
+        <v>7.17875</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A19" s="3"/>
       <c r="F19" s="5"/>
       <c r="I19" s="3"/>
-      <c r="J19" s="1"/>
+      <c r="J19" s="5"/>
       <c r="K19" s="1"/>
       <c r="L19" s="1"/>
       <c r="M19" s="1"/>
       <c r="N19" s="5"/>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="Q19" s="3"/>
+      <c r="R19" s="5"/>
+      <c r="S19" s="1"/>
+      <c r="T19" s="1"/>
+      <c r="U19" s="1"/>
+      <c r="V19" s="5"/>
+    </row>
+    <row r="20" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A20" s="3" t="s">
         <v>22</v>
       </c>
@@ -989,16 +1272,31 @@
       <c r="I20" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="J20" s="1"/>
+      <c r="J20" s="5">
+        <v>25.582000000000001</v>
+      </c>
       <c r="K20" s="1"/>
       <c r="L20" s="1"/>
       <c r="M20" s="1"/>
       <c r="N20" s="5">
-        <f t="shared" ref="N20:N25" si="2">SUM(J20:M20)/4</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.45">
+        <f t="shared" ref="N20" si="3">SUM(J20:M20)/4</f>
+        <v>6.3955000000000002</v>
+      </c>
+      <c r="Q20" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="R20" s="5">
+        <v>25.606999999999999</v>
+      </c>
+      <c r="S20" s="1"/>
+      <c r="T20" s="1"/>
+      <c r="U20" s="1"/>
+      <c r="V20" s="5">
+        <f t="shared" ref="V20" si="4">SUM(R20:U20)/4</f>
+        <v>6.4017499999999998</v>
+      </c>
+    </row>
+    <row r="21" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A21" s="3" t="s">
         <v>23</v>
       </c>
@@ -1012,7 +1310,9 @@
       <c r="I21" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="J21" s="1"/>
+      <c r="J21" s="1" t="s">
+        <v>30</v>
+      </c>
       <c r="K21" s="1"/>
       <c r="L21" s="1"/>
       <c r="M21" s="1"/>
@@ -1020,8 +1320,21 @@
         <f>SUM(J21:M21)/4</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="Q21" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="R21" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="S21" s="1"/>
+      <c r="T21" s="1"/>
+      <c r="U21" s="1"/>
+      <c r="V21" s="5">
+        <f>SUM(R21:U21)/4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A22" s="3" t="s">
         <v>24</v>
       </c>
@@ -1035,24 +1348,44 @@
       <c r="I22" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="J22" s="1"/>
+      <c r="J22" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="K22" s="1"/>
       <c r="L22" s="1"/>
       <c r="M22" s="1"/>
       <c r="N22" s="5">
-        <f t="shared" ref="N22:N25" si="3">SUM(J22:M22)/4</f>
+        <f t="shared" ref="N22" si="5">SUM(J22:M22)/4</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="Q22" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="R22" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="S22" s="1"/>
+      <c r="T22" s="1"/>
+      <c r="U22" s="1"/>
+      <c r="V22" s="5">
+        <f t="shared" ref="V22" si="6">SUM(R22:U22)/4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:22" x14ac:dyDescent="0.45">
       <c r="F23" s="5"/>
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
       <c r="L23" s="1"/>
       <c r="M23" s="1"/>
       <c r="N23" s="5"/>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="R23" s="1"/>
+      <c r="S23" s="1"/>
+      <c r="T23" s="1"/>
+      <c r="U23" s="1"/>
+      <c r="V23" s="5"/>
+    </row>
+    <row r="24" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A24" s="3" t="s">
         <v>25</v>
       </c>
@@ -1066,18 +1399,31 @@
       <c r="I24" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="J24" s="1">
-        <v>0.13900000000000001</v>
+      <c r="J24" s="5">
+        <v>2.839</v>
       </c>
       <c r="K24" s="1"/>
       <c r="L24" s="1"/>
       <c r="M24" s="1"/>
       <c r="N24" s="5">
-        <f t="shared" ref="N24:N25" si="4">SUM(J24:M24)/4</f>
-        <v>3.4750000000000003E-2</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.45">
+        <f>SUM(J24:M24)/4</f>
+        <v>0.70974999999999999</v>
+      </c>
+      <c r="Q24" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="R24" s="5">
+        <v>4.8849999999999998</v>
+      </c>
+      <c r="S24" s="1"/>
+      <c r="T24" s="1"/>
+      <c r="U24" s="1"/>
+      <c r="V24" s="5">
+        <f>SUM(R24:U24)/4</f>
+        <v>1.2212499999999999</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22" x14ac:dyDescent="0.45">
       <c r="A25" s="3" t="s">
         <v>26</v>
       </c>
@@ -1091,21 +1437,35 @@
       <c r="I25" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="J25" s="1">
-        <v>0.30399999999999999</v>
+      <c r="J25" s="5">
+        <v>3.2320000000000002</v>
       </c>
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
       <c r="M25" s="1"/>
       <c r="N25" s="5">
-        <f t="shared" si="4"/>
-        <v>7.5999999999999998E-2</v>
+        <f t="shared" ref="N24:N25" si="7">SUM(J25:M25)/4</f>
+        <v>0.80800000000000005</v>
+      </c>
+      <c r="Q25" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="R25" s="5">
+        <v>5.532</v>
+      </c>
+      <c r="S25" s="1"/>
+      <c r="T25" s="1"/>
+      <c r="U25" s="1"/>
+      <c r="V25" s="5">
+        <f t="shared" ref="V25" si="8">SUM(R25:U25)/4</f>
+        <v>1.383</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="I1:N1"/>
+    <mergeCell ref="Q1:V1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Con mis datos, pero me faltan un par que intentaré hacer en cuanto regrese a casa
</commit_message>
<xml_diff>
--- a/Claudia/tiempos_MHN.xlsx
+++ b/Claudia/tiempos_MHN.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\claud_rjfw4ak\Documents\GitHub\EvAM-Tools\Claudia\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c5dbecc73b6fc60e/Documentos/GitHub/EvamTools_grupo/Claudia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFBA30C5-D7AD-4438-9938-6F28E46CF7E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="64" documentId="13_ncr:1_{BFBA30C5-D7AD-4438-9938-6F28E46CF7E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F2346CD7-326C-4002-A87A-FC1B20FDCF44}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{FDD89A57-F735-49B2-B076-DD48DEACFA57}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{FDD89A57-F735-49B2-B076-DD48DEACFA57}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="39">
   <si>
     <t>Claudia</t>
   </si>
@@ -147,6 +147,12 @@
   </si>
   <si>
     <t>4m 17,4</t>
+  </si>
+  <si>
+    <t>6m 4,6</t>
+  </si>
+  <si>
+    <t>8m 41.9</t>
   </si>
 </sst>
 </file>
@@ -566,19 +572,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BEEB152-16CF-4E65-B7F1-9FCE82C9BF13}">
   <dimension ref="A1:V27"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="39.3984375" customWidth="1"/>
+    <col min="1" max="1" width="39.44140625" customWidth="1"/>
     <col min="2" max="5" width="10.6640625" style="1"/>
-    <col min="6" max="6" width="12.53125" customWidth="1"/>
-    <col min="9" max="9" width="39.19921875" customWidth="1"/>
-    <col min="13" max="13" width="9.53125" customWidth="1"/>
-    <col min="14" max="14" width="12.46484375" customWidth="1"/>
-    <col min="17" max="17" width="39.46484375" customWidth="1"/>
-    <col min="22" max="22" width="25.46484375" customWidth="1"/>
+    <col min="6" max="6" width="12.5546875" customWidth="1"/>
+    <col min="9" max="9" width="39.21875" customWidth="1"/>
+    <col min="13" max="13" width="9.5546875" customWidth="1"/>
+    <col min="14" max="14" width="12.44140625" customWidth="1"/>
+    <col min="17" max="17" width="39.44140625" customWidth="1"/>
+    <col min="22" max="22" width="25.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:22" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
         <v>21</v>
       </c>
@@ -604,7 +610,7 @@
       <c r="U1" s="7"/>
       <c r="V1" s="7"/>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="1" t="s">
         <v>0</v>
@@ -654,7 +660,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>5</v>
       </c>
@@ -664,9 +670,12 @@
       <c r="C3" s="1">
         <v>0.23200000000000001</v>
       </c>
+      <c r="E3" s="1">
+        <v>0.33100000000000002</v>
+      </c>
       <c r="F3" s="3">
         <f>SUM(B3:E3)/4</f>
-        <v>0.36275000000000002</v>
+        <v>0.44550000000000001</v>
       </c>
       <c r="I3" s="4" t="s">
         <v>5</v>
@@ -678,10 +687,12 @@
         <v>28.253</v>
       </c>
       <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
+      <c r="M3" s="1">
+        <v>50.872</v>
+      </c>
       <c r="N3" s="3">
         <f>SUM(J3:M3)/4</f>
-        <v>20.103749999999998</v>
+        <v>32.821749999999994</v>
       </c>
       <c r="Q3" s="4" t="s">
         <v>5</v>
@@ -693,13 +704,15 @@
         <v>36.085999999999999</v>
       </c>
       <c r="T3" s="1"/>
-      <c r="U3" s="1"/>
+      <c r="U3" s="1">
+        <v>53.48</v>
+      </c>
       <c r="V3" s="3">
         <f>SUM(R3:U3)/4</f>
-        <v>26.393000000000001</v>
-      </c>
-    </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.45">
+        <v>39.762999999999998</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
@@ -709,9 +722,12 @@
       <c r="C4" s="1">
         <v>0.129</v>
       </c>
+      <c r="E4" s="1">
+        <v>0.13600000000000001</v>
+      </c>
       <c r="F4" s="3">
         <f t="shared" ref="F4:F25" si="0">SUM(B4:E4)/4</f>
-        <v>6.275E-2</v>
+        <v>9.6750000000000003E-2</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>6</v>
@@ -723,10 +739,12 @@
         <v>28.49</v>
       </c>
       <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
+      <c r="M4" s="1">
+        <v>57.512999999999998</v>
+      </c>
       <c r="N4" s="3">
         <f t="shared" ref="N4:N18" si="1">SUM(J4:M4)/4</f>
-        <v>13.553000000000001</v>
+        <v>27.931249999999999</v>
       </c>
       <c r="Q4" s="4" t="s">
         <v>6</v>
@@ -738,13 +756,15 @@
         <v>30.312999999999999</v>
       </c>
       <c r="T4" s="1"/>
-      <c r="U4" s="1"/>
+      <c r="U4" s="1">
+        <v>53.237000000000002</v>
+      </c>
       <c r="V4" s="3">
         <f t="shared" ref="V4:V18" si="2">SUM(R4:U4)/4</f>
-        <v>14.3675</v>
-      </c>
-    </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.45">
+        <v>27.676749999999998</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>7</v>
       </c>
@@ -754,9 +774,12 @@
       <c r="C5" s="1">
         <v>0.111</v>
       </c>
+      <c r="E5" s="1">
+        <v>0.14599999999999999</v>
+      </c>
       <c r="F5" s="3">
         <f t="shared" si="0"/>
-        <v>4.1750000000000002E-2</v>
+        <v>7.825E-2</v>
       </c>
       <c r="I5" s="5" t="s">
         <v>7</v>
@@ -768,10 +791,12 @@
         <v>26.934000000000001</v>
       </c>
       <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
+      <c r="M5" s="1">
+        <v>49.798000000000002</v>
+      </c>
       <c r="N5" s="3">
         <f t="shared" si="1"/>
-        <v>12.955</v>
+        <v>25.404499999999999</v>
       </c>
       <c r="Q5" s="5" t="s">
         <v>7</v>
@@ -783,13 +808,15 @@
         <v>30.536999999999999</v>
       </c>
       <c r="T5" s="1"/>
-      <c r="U5" s="1"/>
+      <c r="U5" s="1">
+        <v>54.34</v>
+      </c>
       <c r="V5" s="3">
         <f t="shared" si="2"/>
-        <v>14.087250000000001</v>
-      </c>
-    </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.45">
+        <v>27.672250000000002</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>8</v>
       </c>
@@ -799,9 +826,12 @@
       <c r="C6" s="1">
         <v>9.9000000000000005E-2</v>
       </c>
+      <c r="E6" s="1">
+        <v>0.188</v>
+      </c>
       <c r="F6" s="3">
         <f t="shared" si="0"/>
-        <v>4.2749999999999996E-2</v>
+        <v>8.9749999999999996E-2</v>
       </c>
       <c r="I6" s="5" t="s">
         <v>8</v>
@@ -813,10 +843,12 @@
         <v>27.312999999999999</v>
       </c>
       <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
+      <c r="M6" s="1">
+        <v>49.689</v>
+      </c>
       <c r="N6" s="3">
         <f t="shared" si="1"/>
-        <v>12.288</v>
+        <v>24.710250000000002</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>8</v>
@@ -828,13 +860,15 @@
         <v>30.887</v>
       </c>
       <c r="T6" s="1"/>
-      <c r="U6" s="1"/>
+      <c r="U6" s="1">
+        <v>49.844999999999999</v>
+      </c>
       <c r="V6" s="3">
         <f t="shared" si="2"/>
-        <v>13.763249999999999</v>
-      </c>
-    </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.45">
+        <v>26.224499999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>9</v>
       </c>
@@ -844,9 +878,12 @@
       <c r="C7" s="1">
         <v>0.08</v>
       </c>
+      <c r="E7" s="1">
+        <v>0.28299999999999997</v>
+      </c>
       <c r="F7" s="3">
         <f t="shared" si="0"/>
-        <v>3.9750000000000001E-2</v>
+        <v>0.11049999999999999</v>
       </c>
       <c r="I7" s="5" t="s">
         <v>9</v>
@@ -858,10 +895,12 @@
         <v>28.965</v>
       </c>
       <c r="L7" s="1"/>
-      <c r="M7" s="1"/>
+      <c r="M7" s="1">
+        <v>52.228999999999999</v>
+      </c>
       <c r="N7" s="3">
         <f t="shared" si="1"/>
-        <v>13.135249999999999</v>
+        <v>26.192499999999999</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>9</v>
@@ -873,13 +912,15 @@
         <v>29.256</v>
       </c>
       <c r="T7" s="1"/>
-      <c r="U7" s="1"/>
+      <c r="U7" s="1">
+        <v>59.316000000000003</v>
+      </c>
       <c r="V7" s="3">
         <f t="shared" si="2"/>
-        <v>14.029250000000001</v>
-      </c>
-    </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.45">
+        <v>28.858250000000002</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>10</v>
       </c>
@@ -889,9 +930,12 @@
       <c r="C8" s="1">
         <v>8.5999999999999993E-2</v>
       </c>
+      <c r="E8" s="1">
+        <v>0.17799999999999999</v>
+      </c>
       <c r="F8" s="3">
         <f t="shared" si="0"/>
-        <v>4.7750000000000001E-2</v>
+        <v>9.2249999999999999E-2</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>10</v>
@@ -903,10 +947,12 @@
         <v>26.577000000000002</v>
       </c>
       <c r="L8" s="1"/>
-      <c r="M8" s="1"/>
+      <c r="M8" s="1">
+        <v>51.777000000000001</v>
+      </c>
       <c r="N8" s="3">
         <f t="shared" si="1"/>
-        <v>11.679</v>
+        <v>24.623249999999999</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>10</v>
@@ -918,13 +964,15 @@
         <v>32.151000000000003</v>
       </c>
       <c r="T8" s="1"/>
-      <c r="U8" s="1"/>
+      <c r="U8" s="1">
+        <v>61.362000000000002</v>
+      </c>
       <c r="V8" s="3">
         <f t="shared" si="2"/>
-        <v>14.7685</v>
-      </c>
-    </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.45">
+        <v>30.109000000000002</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>11</v>
       </c>
@@ -934,9 +982,12 @@
       <c r="C9" s="1">
         <v>9.2999999999999999E-2</v>
       </c>
+      <c r="E9" s="1">
+        <v>0.35299999999999998</v>
+      </c>
       <c r="F9" s="3">
         <f t="shared" si="0"/>
-        <v>4.8500000000000001E-2</v>
+        <v>0.13674999999999998</v>
       </c>
       <c r="I9" s="5" t="s">
         <v>11</v>
@@ -948,10 +999,12 @@
         <v>26.625</v>
       </c>
       <c r="L9" s="1"/>
-      <c r="M9" s="1"/>
+      <c r="M9" s="1">
+        <v>52.207999999999998</v>
+      </c>
       <c r="N9" s="3">
         <f t="shared" si="1"/>
-        <v>13.017749999999999</v>
+        <v>26.069749999999999</v>
       </c>
       <c r="Q9" s="5" t="s">
         <v>11</v>
@@ -963,13 +1016,15 @@
         <v>39.572000000000003</v>
       </c>
       <c r="T9" s="1"/>
-      <c r="U9" s="1"/>
+      <c r="U9" s="1">
+        <v>48.871000000000002</v>
+      </c>
       <c r="V9" s="3">
         <f t="shared" si="2"/>
-        <v>16.860250000000001</v>
-      </c>
-    </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.45">
+        <v>29.078000000000003</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>12</v>
       </c>
@@ -978,6 +1033,9 @@
       </c>
       <c r="C10" s="1">
         <v>7.3999999999999996E-2</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>29</v>
       </c>
       <c r="F10" s="3">
         <f t="shared" si="0"/>
@@ -993,7 +1051,9 @@
         <v>27.991</v>
       </c>
       <c r="L10" s="1"/>
-      <c r="M10" s="1"/>
+      <c r="M10" t="s">
+        <v>29</v>
+      </c>
       <c r="N10" s="3">
         <f t="shared" si="1"/>
         <v>13.137</v>
@@ -1008,13 +1068,15 @@
         <v>31.692</v>
       </c>
       <c r="T10" s="1"/>
-      <c r="U10" s="1"/>
+      <c r="U10" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="V10" s="3">
         <f t="shared" si="2"/>
         <v>14.831</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>13</v>
       </c>
@@ -1022,6 +1084,9 @@
         <v>0.115</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="3">
@@ -1038,9 +1103,11 @@
         <v>29</v>
       </c>
       <c r="L11" s="1"/>
-      <c r="M11" s="1"/>
+      <c r="M11" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="N11" s="3">
-        <f t="shared" si="1"/>
+        <f>SUM(J11:M11)/4</f>
         <v>6.1202500000000004</v>
       </c>
       <c r="Q11" s="5" t="s">
@@ -1053,13 +1120,15 @@
         <v>29</v>
       </c>
       <c r="T11" s="1"/>
-      <c r="U11" s="1"/>
+      <c r="U11" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="V11" s="3">
         <f t="shared" si="2"/>
         <v>7.0685000000000002</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>14</v>
       </c>
@@ -1067,6 +1136,9 @@
         <v>7.2999999999999995E-2</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>29</v>
       </c>
       <c r="F12" s="3">
@@ -1083,7 +1155,9 @@
         <v>29</v>
       </c>
       <c r="L12" s="1"/>
-      <c r="M12" s="1"/>
+      <c r="M12" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="N12" s="3">
         <f t="shared" si="1"/>
         <v>6.282</v>
@@ -1098,13 +1172,15 @@
         <v>29</v>
       </c>
       <c r="T12" s="1"/>
-      <c r="U12" s="1"/>
+      <c r="U12" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="V12" s="3">
         <f t="shared" si="2"/>
         <v>6.3635000000000002</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>15</v>
       </c>
@@ -1112,6 +1188,9 @@
         <v>0.11600000000000001</v>
       </c>
       <c r="C13" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>29</v>
       </c>
       <c r="F13" s="3">
@@ -1128,7 +1207,9 @@
         <v>29</v>
       </c>
       <c r="L13" s="1"/>
-      <c r="M13" s="1"/>
+      <c r="M13" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="N13" s="3">
         <f t="shared" si="1"/>
         <v>5.8237500000000004</v>
@@ -1143,13 +1224,15 @@
         <v>29</v>
       </c>
       <c r="T13" s="1"/>
-      <c r="U13" s="1"/>
+      <c r="U13" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="V13" s="3">
         <f t="shared" si="2"/>
         <v>7.2297500000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>16</v>
       </c>
@@ -1157,6 +1240,9 @@
         <v>0.11</v>
       </c>
       <c r="C14" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E14" s="1" t="s">
         <v>29</v>
       </c>
       <c r="F14" s="3">
@@ -1173,7 +1259,9 @@
         <v>29</v>
       </c>
       <c r="L14" s="1"/>
-      <c r="M14" s="1"/>
+      <c r="M14" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="N14" s="3">
         <f t="shared" si="1"/>
         <v>6.1559999999999997</v>
@@ -1188,13 +1276,15 @@
         <v>29</v>
       </c>
       <c r="T14" s="1"/>
-      <c r="U14" s="1"/>
+      <c r="U14" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="V14" s="3">
         <f t="shared" si="2"/>
         <v>7.1267500000000004</v>
       </c>
     </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>17</v>
       </c>
@@ -1202,6 +1292,9 @@
         <v>0.112</v>
       </c>
       <c r="C15" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>29</v>
       </c>
       <c r="F15" s="3">
@@ -1218,7 +1311,9 @@
         <v>29</v>
       </c>
       <c r="L15" s="1"/>
-      <c r="M15" s="1"/>
+      <c r="M15" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="N15" s="3">
         <f t="shared" si="1"/>
         <v>6.35825</v>
@@ -1233,13 +1328,15 @@
         <v>29</v>
       </c>
       <c r="T15" s="1"/>
-      <c r="U15" s="1"/>
+      <c r="U15" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="V15" s="3">
         <f t="shared" si="2"/>
         <v>6.5754999999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>18</v>
       </c>
@@ -1247,6 +1344,9 @@
         <v>0.12</v>
       </c>
       <c r="C16" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>29</v>
       </c>
       <c r="F16" s="3">
@@ -1263,7 +1363,9 @@
         <v>29</v>
       </c>
       <c r="L16" s="1"/>
-      <c r="M16" s="1"/>
+      <c r="M16" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="N16" s="3">
         <f t="shared" si="1"/>
         <v>5.3979999999999997</v>
@@ -1278,13 +1380,15 @@
         <v>29</v>
       </c>
       <c r="T16" s="1"/>
-      <c r="U16" s="1"/>
+      <c r="U16" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="V16" s="3">
         <f t="shared" si="2"/>
         <v>7.2442500000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>19</v>
       </c>
@@ -1292,6 +1396,9 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="C17" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>29</v>
       </c>
       <c r="F17" s="3">
@@ -1308,7 +1415,9 @@
         <v>29</v>
       </c>
       <c r="L17" s="1"/>
-      <c r="M17" s="1"/>
+      <c r="M17" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="N17" s="3">
         <f t="shared" si="1"/>
         <v>5.4037499999999996</v>
@@ -1323,13 +1432,15 @@
         <v>29</v>
       </c>
       <c r="T17" s="1"/>
-      <c r="U17" s="1"/>
+      <c r="U17" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="V17" s="3">
         <f t="shared" si="2"/>
         <v>6.9260000000000002</v>
       </c>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>20</v>
       </c>
@@ -1337,6 +1448,9 @@
         <v>0.11600000000000001</v>
       </c>
       <c r="C18" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>29</v>
       </c>
       <c r="F18" s="3">
@@ -1353,7 +1467,9 @@
         <v>29</v>
       </c>
       <c r="L18" s="1"/>
-      <c r="M18" s="1"/>
+      <c r="M18" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="N18" s="3">
         <f t="shared" si="1"/>
         <v>5.9974999999999996</v>
@@ -1368,13 +1484,15 @@
         <v>29</v>
       </c>
       <c r="T18" s="1"/>
-      <c r="U18" s="1"/>
+      <c r="U18" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="V18" s="3">
         <f t="shared" si="2"/>
         <v>7.17875</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
       <c r="F19" s="3"/>
       <c r="I19" s="5"/>
@@ -1390,7 +1508,7 @@
       <c r="U19" s="1"/>
       <c r="V19" s="3"/>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>22</v>
       </c>
@@ -1400,9 +1518,12 @@
       <c r="C20" s="1">
         <v>9.0999999999999998E-2</v>
       </c>
+      <c r="E20" s="1">
+        <v>2.1000000000000001E-2</v>
+      </c>
       <c r="F20" s="3">
         <f t="shared" si="0"/>
-        <v>5.7500000000000002E-2</v>
+        <v>6.275E-2</v>
       </c>
       <c r="I20" s="5" t="s">
         <v>22</v>
@@ -1414,10 +1535,12 @@
         <v>29.306000000000001</v>
       </c>
       <c r="L20" s="1"/>
-      <c r="M20" s="1"/>
+      <c r="M20" s="1">
+        <v>52.137999999999998</v>
+      </c>
       <c r="N20" s="3">
         <f t="shared" ref="N20" si="3">SUM(J20:M20)/4</f>
-        <v>13.722000000000001</v>
+        <v>26.756500000000003</v>
       </c>
       <c r="Q20" s="5" t="s">
         <v>22</v>
@@ -1429,13 +1552,15 @@
         <v>33.119999999999997</v>
       </c>
       <c r="T20" s="1"/>
-      <c r="U20" s="1"/>
+      <c r="U20" s="1">
+        <v>54.359000000000002</v>
+      </c>
       <c r="V20" s="3">
         <f t="shared" ref="V20" si="4">SUM(R20:U20)/4</f>
-        <v>14.681749999999999</v>
-      </c>
-    </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.45">
+        <v>28.2715</v>
+      </c>
+    </row>
+    <row r="21" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>23</v>
       </c>
@@ -1480,7 +1605,7 @@
         <v>35.83</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>24</v>
       </c>
@@ -1525,7 +1650,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A23" s="6"/>
       <c r="F23" s="3"/>
       <c r="I23" s="6"/>
@@ -1541,7 +1666,7 @@
       <c r="U23" s="1"/>
       <c r="V23" s="3"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>25</v>
       </c>
@@ -1551,9 +1676,12 @@
       <c r="C24" s="1" t="s">
         <v>34</v>
       </c>
+      <c r="E24" s="1">
+        <v>2.5</v>
+      </c>
       <c r="F24" s="3">
-        <f t="shared" si="0"/>
-        <v>1.0749999999999999E-2</v>
+        <f>SUM(B24:E24)/4</f>
+        <v>0.63575000000000004</v>
       </c>
       <c r="I24" s="5" t="s">
         <v>25</v>
@@ -1564,11 +1692,12 @@
       <c r="K24" s="1">
         <v>18.8</v>
       </c>
-      <c r="L24" s="1"/>
-      <c r="M24" s="1"/>
+      <c r="M24" s="1">
+        <v>2.6</v>
+      </c>
       <c r="N24" s="3">
         <f>SUM(J24:M24)/4</f>
-        <v>5.4097499999999998</v>
+        <v>6.0597500000000002</v>
       </c>
       <c r="Q24" s="5" t="s">
         <v>25</v>
@@ -1580,13 +1709,15 @@
         <v>12.5</v>
       </c>
       <c r="T24" s="1"/>
-      <c r="U24" s="1"/>
+      <c r="U24">
+        <v>33.4</v>
+      </c>
       <c r="V24" s="3">
         <f>SUM(R24:U24)/4</f>
-        <v>4.3462499999999995</v>
-      </c>
-    </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.45">
+        <v>12.696249999999999</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>26</v>
       </c>
@@ -1596,9 +1727,12 @@
       <c r="C25" s="1" t="s">
         <v>34</v>
       </c>
+      <c r="E25" s="1">
+        <v>3.4</v>
+      </c>
       <c r="F25" s="3">
-        <f t="shared" si="0"/>
-        <v>9.75E-3</v>
+        <f>SUM(B25:E25)/4</f>
+        <v>0.85975000000000001</v>
       </c>
       <c r="I25" s="5" t="s">
         <v>26</v>
@@ -1609,11 +1743,12 @@
       <c r="K25" s="1">
         <v>4.5999999999999996</v>
       </c>
-      <c r="L25" s="1"/>
-      <c r="M25" s="1"/>
+      <c r="M25" s="1">
+        <v>2.7</v>
+      </c>
       <c r="N25" s="3">
-        <f t="shared" ref="N25" si="7">SUM(J25:M25)/4</f>
-        <v>1.958</v>
+        <f>SUM(J25:M25)/4</f>
+        <v>2.633</v>
       </c>
       <c r="Q25" s="5" t="s">
         <v>26</v>
@@ -1625,50 +1760,70 @@
         <v>19.3</v>
       </c>
       <c r="T25" s="1"/>
-      <c r="U25" s="1"/>
+      <c r="U25">
+        <v>37.700000000000003</v>
+      </c>
       <c r="V25" s="3">
-        <f t="shared" ref="V25" si="8">SUM(R25:U25)/4</f>
-        <v>6.2080000000000002</v>
-      </c>
-    </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.45">
+        <f t="shared" ref="V25" si="7">SUM(R25:U25)/4</f>
+        <v>15.633000000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>32</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>34</v>
       </c>
+      <c r="E26">
+        <v>43.3</v>
+      </c>
       <c r="I26" s="5" t="s">
         <v>32</v>
       </c>
       <c r="K26" s="1">
         <v>22.9</v>
       </c>
+      <c r="M26" s="1">
+        <v>34.1</v>
+      </c>
       <c r="Q26" s="5" t="s">
         <v>32</v>
       </c>
       <c r="S26" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="U26" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="27" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>33</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>34</v>
       </c>
+      <c r="E27" s="1">
+        <v>45.6</v>
+      </c>
       <c r="I27" s="5" t="s">
         <v>33</v>
       </c>
       <c r="K27" s="1">
         <v>27.5</v>
       </c>
+      <c r="M27" s="1">
+        <v>45.3</v>
+      </c>
       <c r="Q27" s="5" t="s">
         <v>33</v>
       </c>
       <c r="S27" s="1" t="s">
         <v>36</v>
+      </c>
+      <c r="U27" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tiempos de shiny pero solo BRCA
</commit_message>
<xml_diff>
--- a/Claudia/tiempos_MHN.xlsx
+++ b/Claudia/tiempos_MHN.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tania\Documents\GitHub\EvAM-Tools\Claudia\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c5dbecc73b6fc60e/Documentos/GitHub/EvamTools_grupo/Claudia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92038662-50C2-4E7F-9144-B0E94BF2B232}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{92038662-50C2-4E7F-9144-B0E94BF2B232}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24CAAFC5-156B-497D-A589-22A4810FC8F2}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{FDD89A57-F735-49B2-B076-DD48DEACFA57}"/>
   </bookViews>
@@ -1779,9 +1779,12 @@
       <c r="C21" s="1">
         <v>7.38</v>
       </c>
+      <c r="F21" s="1">
+        <v>3.58</v>
+      </c>
       <c r="G21" s="3">
         <f>SUM(B21:F21)/4</f>
-        <v>2.7050000000000001</v>
+        <v>3.6</v>
       </c>
       <c r="J21" s="5" t="s">
         <v>23</v>
@@ -1824,9 +1827,12 @@
       <c r="C22" s="1">
         <v>18.48</v>
       </c>
+      <c r="F22" s="1">
+        <v>11.41</v>
+      </c>
       <c r="G22" s="3">
         <f t="shared" si="0"/>
-        <v>8.2624999999999993</v>
+        <v>11.114999999999998</v>
       </c>
       <c r="J22" s="5" t="s">
         <v>24</v>

</xml_diff>

<commit_message>
nuevo tiempo para web
</commit_message>
<xml_diff>
--- a/Claudia/tiempos_MHN.xlsx
+++ b/Claudia/tiempos_MHN.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\claud_rjfw4ak\Documents\GitHub\EvAM-Tools\Claudia\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sandra\Documents\GitHub\EvAM-Tools\Claudia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88E24DFF-46BF-4F6A-8B8B-AE7E8F92EF75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F92F37C5-7660-4C67-B34C-5DCE03411371}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{FDD89A57-F735-49B2-B076-DD48DEACFA57}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{FDD89A57-F735-49B2-B076-DD48DEACFA57}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="49">
   <si>
     <t>Claudia</t>
   </si>
@@ -180,6 +180,9 @@
   </si>
   <si>
     <t>Claudia 2</t>
+  </si>
+  <si>
+    <t>2m 15</t>
   </si>
 </sst>
 </file>
@@ -608,21 +611,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BEEB152-16CF-4E65-B7F1-9FCE82C9BF13}">
   <dimension ref="A1:X27"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="49" customWidth="1"/>
     <col min="2" max="5" width="10.6640625" style="1"/>
-    <col min="6" max="6" width="11.53125" style="1"/>
+    <col min="6" max="6" width="11.5546875" style="1"/>
     <col min="7" max="7" width="10.6640625" style="1"/>
-    <col min="8" max="8" width="12.53125" customWidth="1"/>
-    <col min="11" max="11" width="39.19921875" customWidth="1"/>
-    <col min="15" max="15" width="9.53125" customWidth="1"/>
-    <col min="16" max="16" width="12.46484375" customWidth="1"/>
-    <col min="19" max="19" width="39.46484375" customWidth="1"/>
-    <col min="24" max="24" width="25.46484375" customWidth="1"/>
+    <col min="8" max="8" width="12.5546875" customWidth="1"/>
+    <col min="11" max="11" width="39.21875" customWidth="1"/>
+    <col min="15" max="15" width="9.5546875" customWidth="1"/>
+    <col min="16" max="16" width="12.44140625" customWidth="1"/>
+    <col min="19" max="19" width="39.44140625" customWidth="1"/>
+    <col min="24" max="24" width="25.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="18" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:24" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="8" t="s">
         <v>21</v>
       </c>
@@ -650,7 +653,7 @@
       <c r="W1" s="8"/>
       <c r="X1" s="8"/>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="1" t="s">
         <v>0</v>
@@ -706,7 +709,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>5</v>
       </c>
@@ -771,7 +774,7 @@
         <v>47.110749999999996</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
@@ -836,7 +839,7 @@
         <v>34.947749999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>7</v>
       </c>
@@ -901,7 +904,7 @@
         <v>34.843000000000004</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>8</v>
       </c>
@@ -966,7 +969,7 @@
         <v>33.512749999999997</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>9</v>
       </c>
@@ -1031,7 +1034,7 @@
         <v>36.071750000000002</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>10</v>
       </c>
@@ -1096,7 +1099,7 @@
         <v>37.441000000000003</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>11</v>
       </c>
@@ -1161,7 +1164,7 @@
         <v>36.429250000000003</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>12</v>
       </c>
@@ -1226,7 +1229,7 @@
         <v>22.208749999999998</v>
       </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>13</v>
       </c>
@@ -1291,7 +1294,7 @@
         <v>14.27275</v>
       </c>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>14</v>
       </c>
@@ -1356,7 +1359,7 @@
         <v>13.5535</v>
       </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>15</v>
       </c>
@@ -1421,7 +1424,7 @@
         <v>14.46</v>
       </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>16</v>
       </c>
@@ -1486,7 +1489,7 @@
         <v>14.418749999999999</v>
       </c>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>17</v>
       </c>
@@ -1551,7 +1554,7 @@
         <v>6.5754999999999999</v>
       </c>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>18</v>
       </c>
@@ -1616,7 +1619,7 @@
         <v>7.2442500000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>19</v>
       </c>
@@ -1681,7 +1684,7 @@
         <v>6.9260000000000002</v>
       </c>
     </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>20</v>
       </c>
@@ -1746,7 +1749,7 @@
         <v>7.17875</v>
       </c>
     </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
       <c r="H19" s="3"/>
       <c r="K19" s="5"/>
@@ -1762,7 +1765,7 @@
       <c r="W19" s="1"/>
       <c r="X19" s="3"/>
     </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>22</v>
       </c>
@@ -1824,7 +1827,7 @@
         <v>35.537999999999997</v>
       </c>
     </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>23</v>
       </c>
@@ -1847,14 +1850,14 @@
       <c r="L21" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="M21" s="1">
-        <v>5.52</v>
+      <c r="M21" s="1" t="s">
+        <v>48</v>
       </c>
       <c r="N21" s="1"/>
       <c r="O21" s="1"/>
       <c r="P21" s="3">
         <f>SUM(L21:O21)/4</f>
-        <v>1.38</v>
+        <v>0</v>
       </c>
       <c r="S21" s="5" t="s">
         <v>23</v>
@@ -1872,7 +1875,7 @@
         <v>35.83</v>
       </c>
     </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>24</v>
       </c>
@@ -1895,14 +1898,12 @@
       <c r="L22" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="M22" s="1">
-        <v>11.11</v>
-      </c>
+      <c r="M22" s="1"/>
       <c r="N22" s="1"/>
       <c r="O22" s="1"/>
       <c r="P22" s="3">
         <f t="shared" ref="P22" si="5">SUM(L22:O22)/4</f>
-        <v>2.7774999999999999</v>
+        <v>0</v>
       </c>
       <c r="S22" s="5" t="s">
         <v>24</v>
@@ -1920,7 +1921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A23" s="6"/>
       <c r="H23" s="3"/>
       <c r="K23" s="6"/>
@@ -1936,7 +1937,7 @@
       <c r="W23" s="1"/>
       <c r="X23" s="3"/>
     </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>25</v>
       </c>
@@ -1995,7 +1996,7 @@
         <v>12.696249999999999</v>
       </c>
     </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>26</v>
       </c>
@@ -2054,7 +2055,7 @@
         <v>15.633000000000001</v>
       </c>
     </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>32</v>
       </c>
@@ -2092,7 +2093,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>33</v>
       </c>

</xml_diff>